<commit_message>
Restore D-02 Claude multiple; set force majeure long-stop to 60 days uniformly
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012r6bKnXcJp9a2cyYVk4obL
</commit_message>
<xml_diff>
--- a/skills/contract-review-flagger/references/Start2_Asia_Contract_Standards_UP_05_Oct.xlsx
+++ b/skills/contract-review-flagger/references/Start2_Asia_Contract_Standards_UP_05_Oct.xlsx
@@ -1280,7 +1280,7 @@
       </c>
       <c r="G20" s="8" t="inlineStr">
         <is>
-          <t>If the ability of either party to perform any of its obligations under this Agreement is limited, delayed or prevented in whole or in part by reason of any cause or event beyond the reasonable control of such party, including but without limitation fire, storm, tempest, explosion, accident, breakdown of plant or machinery, strike and/or industrial dispute, war, civil strike or commotion, act of foreign enemy, epidemic, quarantine, health risk, terrorist activity, events of national emergency, hostilities (whether war be declared or not), law or act of or authorised by a government but excluding the inability to meet financial obligations (a "Force Majeure Event"), such party shall be excused, discharged or released without penalty or liability from its obligations under this Agreement to the extent and for the period that such performance is so limited, delayed or prevented PROVIDED that such party shall take all steps reasonably possible to mitigate the losses or damages caused by its failure or delay to perform its obligations under this Agreement. Notwithstanding the foregoing, if the Force Majeure Event exceeds one (1) month in duration, either party shall have the right at any time thereafter during the continuance of such failure or delay, to terminate this Agreement by giving written notice to the other party.</t>
+          <t>If the ability of either party to perform any of its obligations under this Agreement is limited, delayed or prevented in whole or in part by reason of any cause or event beyond the reasonable control of such party, including but without limitation fire, storm, tempest, explosion, accident, breakdown of plant or machinery, strike and/or industrial dispute, war, civil strike or commotion, act of foreign enemy, epidemic, quarantine, health risk, terrorist activity, events of national emergency, hostilities (whether war be declared or not), law or act of or authorised by a government but excluding the inability to meet financial obligations (a "Force Majeure Event"), such party shall be excused, discharged or released without penalty or liability from its obligations under this Agreement to the extent and for the period that such performance is so limited, delayed or prevented PROVIDED that such party shall take all steps reasonably possible to mitigate the losses or damages caused by its failure or delay to perform its obligations under this Agreement. Notwithstanding the foregoing, if the Force Majeure Event exceeds sixty (60) days in duration, either party shall have the right at any time thereafter during the continuance of such failure or delay, to terminate this Agreement by giving written notice to the other party.</t>
         </is>
       </c>
     </row>
@@ -1977,7 +1977,7 @@
       <c r="C20" s="2" t="inlineStr">
         <is>
           <t>18.1 If the ability of either party to perform any of its obligations under this Agreement is limited, delayed or prevented in whole or in part by reason of any cause or event beyond the reasonable control of such party, including but without limitation fire, storm, tempest, explosion, accident, breakdown of plant or machinery, strike and/or industrial dispute, war, civil strike or commotion, act of foreign enemy, epidemic, quarantine, health risk, terrorist activity, events of national emergency, hostilities (whether war be declared or not), law or act of or authorised by a government but excluding the inability to meet financial obligations (a "Force Majeure Event"), such party shall be excused, discharged or released without penalty or liability from its obligations under this Agreement to the extent and for the period that such performance is so limited, delayed or prevented provided that such party shall take all steps reasonably possible to mitigate the losses or damages caused by its failure or delay to perform its obligations under this Agreement. 
-18.2 If a Force Majeure Event under Clause [Force Majeure] continues for more than one (1) month, the Parties shall first discuss in good faith, for up to [14] days, whether to postpone or reschedule the Service instead of terminating this Agreement.
+18.2 If a Force Majeure Event under Clause [Force Majeure] continues for more than sixty (60) days, the Parties shall first discuss in good faith, for up to [14] days, whether to postpone or reschedule the Service instead of terminating this Agreement.
 18.3 If the Parties do not agree to postpone or reschedule within that period, either Party may terminate this Agreement on written notice to the other, without liability, other than for amounts already due under Clause [Cost Recovery on Cancellation].</t>
         </is>
       </c>
@@ -2577,7 +2577,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Not sure</t>
+          <t>(b), 2x total fees as a starting ask. These breach types carry third-party exposure the general cap was not built for.</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -2701,12 +2701,12 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>1 month. The long-stop before either party may terminate for prolonged force majeure is one (1) month, matching the Force majeure reference clause.</t>
+          <t xml:space="preserve">(b), 60 days as a default. Long enough that ordinary short disruptions don't trigger an exit right either side didn't want, short enough that a program stuck for two months has a way out. </t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>1 month. The long-stop before either party may terminate for prolonged force majeure is one (1) month, matching the Force majeure reference clause.</t>
+          <t xml:space="preserve">(b), 60 days as a default. </t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">

</xml_diff>